<commit_message>
Fix: Aggressive PDF space optimization with smart image shrinking to remove blank gaps
</commit_message>
<xml_diff>
--- a/ERP Report/PICS/P1/K.xlsx
+++ b/ERP Report/PICS/P1/K.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SRINIVASU(BNG11531)\ECITY\SNAPSHOT\Jr.SUPER60\22-06-2025_Jr.Super60_NUCLEUS BT_Jee-Adv(2023-P1)_WTA-11_Q. Paper &amp; Key &amp; Sol's\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SRINIVASU(BNG11531)\ECITY\SNAPSHOT\Jr.SUPER60\29-06-2025_Jr.Super60_NUCLEUS BT_Jee-Adv(2022-P1)_WTA-12_Q. Paper &amp; Key &amp; Sol's\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967B9DAA-ED7A-42F4-8765-1227EAC4C065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC79F060-B774-4870-B4AF-04F538A8C03F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="15">
   <si>
     <t>Q_No</t>
   </si>
@@ -46,22 +46,25 @@
     <t>ABC</t>
   </si>
   <si>
-    <t>ACD</t>
-  </si>
-  <si>
-    <t>ABD</t>
+    <t>D</t>
   </si>
   <si>
     <t>AC</t>
   </si>
   <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>BD</t>
+    <t>BCD</t>
   </si>
   <si>
     <t>BC</t>
+  </si>
+  <si>
+    <t>CD</t>
+  </si>
+  <si>
+    <t>AD</t>
+  </si>
+  <si>
+    <t>6.3-6.6</t>
   </si>
 </sst>
 </file>
@@ -1086,7 +1089,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1"/>
@@ -1105,56 +1108,56 @@
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>9</v>
+      <c r="B2" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>10</v>
+      <c r="B3" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>4</v>
+      <c r="B4" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>5</v>
+      <c r="B5" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>11</v>
+      <c r="B6" s="2">
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>5</v>
+      <c r="B7" s="2">
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>2</v>
+      <c r="B8" s="2">
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1162,47 +1165,47 @@
         <v>8</v>
       </c>
       <c r="B9" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="2">
-        <v>13</v>
+      <c r="B10" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="2">
-        <v>50</v>
+      <c r="B11" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="2">
-        <v>100</v>
+      <c r="B12" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" s="2">
-        <v>0</v>
+      <c r="B13" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="2">
-        <v>216</v>
+      <c r="B14" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1218,7 +1221,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1226,7 +1229,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1234,7 +1237,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -1242,30 +1245,30 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>6</v>
+      <c r="B20" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>7</v>
+      <c r="B21" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="2">
         <v>5</v>
       </c>
     </row>
@@ -1273,24 +1276,24 @@
       <c r="A23" s="1">
         <v>22</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>11</v>
+      <c r="B23" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>11</v>
+      <c r="B24" s="2">
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>3</v>
+      <c r="B25" s="2">
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -1298,7 +1301,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
@@ -1306,39 +1309,39 @@
         <v>26</v>
       </c>
       <c r="B27" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>27</v>
       </c>
-      <c r="B28" s="2">
-        <v>6</v>
+      <c r="B28" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>28</v>
       </c>
-      <c r="B29" s="2">
-        <v>0</v>
+      <c r="B29" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>29</v>
       </c>
-      <c r="B30" s="2">
-        <v>3</v>
+      <c r="B30" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>30</v>
       </c>
-      <c r="B31" s="2">
-        <v>2</v>
+      <c r="B31" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -1346,7 +1349,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
@@ -1354,7 +1357,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
@@ -1362,7 +1365,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
@@ -1370,7 +1373,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
@@ -1378,7 +1381,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
@@ -1386,23 +1389,23 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>37</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>10</v>
+      <c r="B38" s="2">
+        <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>38</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>5</v>
+      <c r="B39" s="2">
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
@@ -1410,23 +1413,23 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>40</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>3</v>
+      <c r="B41" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>41</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>5</v>
+      <c r="B42" s="2">
+        <v>25</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
@@ -1434,7 +1437,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="2">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
@@ -1442,7 +1445,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="2">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
@@ -1450,30 +1453,30 @@
         <v>44</v>
       </c>
       <c r="B45" s="2">
-        <v>3</v>
+        <v>160</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>45</v>
       </c>
-      <c r="B46" s="2">
-        <v>3</v>
+      <c r="B46" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>46</v>
       </c>
-      <c r="B47" s="2">
-        <v>4</v>
+      <c r="B47" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>47</v>
       </c>
-      <c r="B48" s="2">
+      <c r="B48" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1482,7 +1485,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
@@ -1490,7 +1493,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
@@ -1506,6 +1509,30 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" s="1">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" s="1">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" s="1">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update: Performance and UI improvements
</commit_message>
<xml_diff>
--- a/ERP Report/PICS/P1/K.xlsx
+++ b/ERP Report/PICS/P1/K.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SRINIVASU(BNG11531)\ECITY\SNAPSHOT\Jr.SUPER60\29-06-2025_Jr.Super60_NUCLEUS BT_Jee-Adv(2022-P1)_WTA-12_Q. Paper &amp; Key &amp; Sol's\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SRINIVASU(BNG11531)\ECITY\SNAPSHOT\Jr.SUPER60\24-08-2025_Jr.Super60_NUCLEUS BT_Jee-Adv(2020-P1)_WTA-19_Q. Paper &amp; Key &amp; Sol's\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC79F060-B774-4870-B4AF-04F538A8C03F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0DF87A-D3E2-4DB3-A99A-157BC28CA5C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="15">
   <si>
     <t>Q_No</t>
   </si>
@@ -46,25 +46,25 @@
     <t>ABC</t>
   </si>
   <si>
+    <t>ACD</t>
+  </si>
+  <si>
+    <t>ABD</t>
+  </si>
+  <si>
     <t>D</t>
   </si>
   <si>
-    <t>AC</t>
+    <t>BD</t>
+  </si>
+  <si>
+    <t>AD</t>
   </si>
   <si>
     <t>BCD</t>
   </si>
   <si>
-    <t>BC</t>
-  </si>
-  <si>
-    <t>CD</t>
-  </si>
-  <si>
-    <t>AD</t>
-  </si>
-  <si>
-    <t>6.3-6.6</t>
+    <t>1.8-2.0</t>
   </si>
 </sst>
 </file>
@@ -1108,64 +1108,64 @@
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
-        <v>4</v>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="2">
-        <v>2</v>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="2">
-        <v>1</v>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="2">
-        <v>2</v>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="2">
-        <v>9</v>
+      <c r="B6" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="2">
-        <v>3</v>
+      <c r="B7" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="2">
-        <v>3</v>
+      <c r="B8" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="2">
-        <v>8</v>
+      <c r="B9" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1173,7 +1173,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1181,7 +1181,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1189,7 +1189,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1197,119 +1197,119 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>7</v>
+      <c r="B14" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>11</v>
+      <c r="B15" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>8</v>
+      <c r="B16" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>3</v>
+      <c r="B17" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>8</v>
+      <c r="B18" s="2">
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>8</v>
+      <c r="B19" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" s="2">
-        <v>5</v>
+      <c r="B20" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="2">
-        <v>8</v>
+      <c r="B21" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>21</v>
       </c>
-      <c r="B22" s="2">
-        <v>5</v>
+      <c r="B22" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>22</v>
       </c>
-      <c r="B23" s="2">
-        <v>5</v>
+      <c r="B23" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>23</v>
       </c>
-      <c r="B24" s="2">
-        <v>6</v>
+      <c r="B24" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>24</v>
       </c>
-      <c r="B25" s="2">
-        <v>6</v>
+      <c r="B25" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>25</v>
       </c>
-      <c r="B26" s="2">
-        <v>8</v>
+      <c r="B26" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>26</v>
       </c>
-      <c r="B27" s="2">
-        <v>2</v>
+      <c r="B27" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
@@ -1325,7 +1325,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
@@ -1333,7 +1333,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
@@ -1341,7 +1341,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -1349,63 +1349,63 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>32</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>13</v>
+      <c r="B33" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>33</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>5</v>
+      <c r="B34" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>34</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>2</v>
+      <c r="B35" s="2">
+        <v>1.2</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>35</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>8</v>
+      <c r="B36" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>36</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>3</v>
+      <c r="B37" s="2">
+        <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>37</v>
       </c>
-      <c r="B38" s="2">
-        <v>3</v>
+      <c r="B38" s="2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>38</v>
       </c>
-      <c r="B39" s="2">
-        <v>7</v>
+      <c r="B39" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
@@ -1413,38 +1413,38 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>40</v>
       </c>
-      <c r="B41" s="2">
-        <v>2</v>
+      <c r="B41" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>41</v>
       </c>
-      <c r="B42" s="2">
-        <v>25</v>
+      <c r="B42" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>42</v>
       </c>
-      <c r="B43" s="2">
-        <v>6</v>
+      <c r="B43" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>43</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1452,8 +1452,8 @@
       <c r="A45" s="1">
         <v>44</v>
       </c>
-      <c r="B45" s="2">
-        <v>160</v>
+      <c r="B45" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
@@ -1461,7 +1461,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
@@ -1469,7 +1469,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
@@ -1477,7 +1477,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -1485,55 +1485,55 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>49</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>6</v>
+      <c r="B50" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>50</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>11</v>
+      <c r="B51" s="2">
+        <v>3</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>51</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>2</v>
+      <c r="B52" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>52</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>2</v>
+      <c r="B53" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>53</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>3</v>
+      <c r="B54" s="2">
+        <v>91</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>54</v>
       </c>
-      <c r="B55" s="2" t="s">
-        <v>5</v>
+      <c r="B55" s="2">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Uptime Robot failure and the Loading...
</commit_message>
<xml_diff>
--- a/ERP Report/PICS/P1/K.xlsx
+++ b/ERP Report/PICS/P1/K.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SRINIVASU(BNG11531)\ECITY\SNAPSHOT\Jr.SUPER60\24-08-2025_Jr.Super60_NUCLEUS BT_Jee-Adv(2020-P1)_WTA-19_Q. Paper &amp; Key &amp; Sol's\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SRINIVASU(BNG11531)\ECITY\SNAPSHOT\Jr.SUPER60\22-06-2025_Jr.Super60_NUCLEUS BT_Jee-Adv(2023-P1)_WTA-11_Q. Paper &amp; Key &amp; Sol's\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0DF87A-D3E2-4DB3-A99A-157BC28CA5C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967B9DAA-ED7A-42F4-8765-1227EAC4C065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="14">
   <si>
     <t>Q_No</t>
   </si>
@@ -52,19 +52,16 @@
     <t>ABD</t>
   </si>
   <si>
+    <t>AC</t>
+  </si>
+  <si>
     <t>D</t>
   </si>
   <si>
     <t>BD</t>
   </si>
   <si>
-    <t>AD</t>
-  </si>
-  <si>
-    <t>BCD</t>
-  </si>
-  <si>
-    <t>1.8-2.0</t>
+    <t>BC</t>
   </si>
 </sst>
 </file>
@@ -1089,7 +1086,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B55"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1"/>
@@ -1109,7 +1106,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1125,7 +1122,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1141,7 +1138,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="27" customHeight="1" x14ac:dyDescent="0.2">
@@ -1149,7 +1146,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1157,47 +1154,47 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>7</v>
+      <c r="B9" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>8</v>
+      <c r="B10" s="2">
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>6</v>
+      <c r="B11" s="2">
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>8</v>
+      <c r="B12" s="2">
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>7</v>
+      <c r="B13" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
@@ -1205,30 +1202,30 @@
         <v>13</v>
       </c>
       <c r="B14" s="2">
-        <v>8</v>
+        <v>216</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="2">
-        <v>2</v>
+      <c r="B15" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="2">
-        <v>4</v>
+      <c r="B16" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="2" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1236,16 +1233,16 @@
       <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" s="2">
-        <v>3</v>
+      <c r="B18" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" s="2">
-        <v>2</v>
+      <c r="B19" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -1253,7 +1250,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -1261,7 +1258,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
@@ -1269,7 +1266,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
@@ -1277,7 +1274,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
@@ -1285,7 +1282,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
@@ -1293,55 +1290,55 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>13</v>
+      <c r="B26" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>9</v>
+      <c r="B27" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>27</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>11</v>
+      <c r="B28" s="2">
+        <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>28</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>13</v>
+      <c r="B29" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>29</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>6</v>
+      <c r="B30" s="2">
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>30</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>6</v>
+      <c r="B31" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -1349,47 +1346,47 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>32</v>
       </c>
-      <c r="B33" s="2">
-        <v>1</v>
+      <c r="B33" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>33</v>
       </c>
-      <c r="B34" s="2">
-        <v>2</v>
+      <c r="B34" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>34</v>
       </c>
-      <c r="B35" s="2">
-        <v>1.2</v>
+      <c r="B35" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>35</v>
       </c>
-      <c r="B36" s="2">
-        <v>2</v>
+      <c r="B36" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>36</v>
       </c>
-      <c r="B37" s="2">
-        <v>6</v>
+      <c r="B37" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
@@ -1397,7 +1394,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
@@ -1405,7 +1402,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
@@ -1436,7 +1433,7 @@
       <c r="A43" s="1">
         <v>42</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="2">
         <v>3</v>
       </c>
     </row>
@@ -1444,40 +1441,40 @@
       <c r="A44" s="1">
         <v>43</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>6</v>
+      <c r="B44" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>44</v>
       </c>
-      <c r="B45" s="2" t="s">
-        <v>11</v>
+      <c r="B45" s="2">
+        <v>3</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>45</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>7</v>
+      <c r="B46" s="2">
+        <v>3</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>46</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>9</v>
+      <c r="B47" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>47</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>6</v>
+      <c r="B48" s="2">
+        <v>8</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -1485,55 +1482,31 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>49</v>
       </c>
-      <c r="B50" s="2">
-        <v>0</v>
+      <c r="B50" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>50</v>
       </c>
-      <c r="B51" s="2">
-        <v>3</v>
+      <c r="B51" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>51</v>
       </c>
-      <c r="B52" s="2">
+      <c r="B52" s="2" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A53" s="1">
-        <v>52</v>
-      </c>
-      <c r="B53" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A54" s="1">
-        <v>53</v>
-      </c>
-      <c r="B54" s="2">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A55" s="1">
-        <v>54</v>
-      </c>
-      <c r="B55" s="2">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>